<commit_message>
UISS: switch off Excel's 'Number Stored as Text' marker on every sheet (FB-102)
clean_uiss_xlsx.py adds ignoredErrors numberStoredAsText to each worksheet (numbering such as '1.'
is text on purpose), so future builds keep it; applied to the 13 UISS of function_list_v2,
including the hand-tidied XD01 (content and layout unchanged).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/uiss/XD04_UISS_Batch_ActualDemandSummarySync.xlsx
+++ b/deliverables/function_list_v2/uiss/XD04_UISS_Batch_ActualDemandSummarySync.xlsx
@@ -11955,6 +11955,9 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.590277777777778" right="0.509722222222222" top="0.865972222222222" bottom="0.39375" header="0.865972222222222" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -17204,6 +17207,9 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.7" bottom="0.25" header="0.6" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -22509,6 +22515,9 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.7" bottom="0.25" header="0.6" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -33023,6 +33032,9 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="48" min="0" max="16383" man="1"/>
   </rowBreaks>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -38097,6 +38109,9 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.7" bottom="0.25" header="0.6" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -43103,6 +43118,9 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.7" bottom="0.25" header="0.6" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -48536,6 +48554,9 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.25" right="0.25" top="0.7" bottom="0.25" header="0.6" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -48927,5 +48948,8 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:XFD1048576" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>